<commit_message>
feat: Enhance scoring rules and race handling by implementing cancellation logic and normalizing driver names
</commit_message>
<xml_diff>
--- a/Formula F1NTA 2026.xlsx
+++ b/Formula F1NTA 2026.xlsx
@@ -1,16 +1,13 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <workbookPr/>
-  <sheets>
-    <sheet state="visible" name="Foglio1" sheetId="1" r:id="rId4"/>
-  </sheets>
-  <definedNames/>
-  <calcPr/>
-</workbook>
+<file path=xl\drawings\drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\persons\person.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="103">
   <si>
     <t xml:space="preserve">    </t>
@@ -363,7 +360,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <fonts count="17">
     <font>
@@ -1298,15 +1295,18 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <workbookPr/>
+  <sheets>
+    <sheet state="visible" name="Foglio1" sheetId="1" r:id="rId4"/>
+  </sheets>
+  <definedNames/>
+  <calcPr/>
+</workbook>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <pageSetUpPr/>
@@ -1945,7 +1945,6 @@
         <v>12</v>
       </c>
       <c r="W11" s="8"/>
-      <c r="X11" s="11"/>
       <c r="Y11" s="34"/>
       <c r="Z11" s="34"/>
       <c r="AA11" s="34"/>
@@ -1962,6 +1961,11 @@
       <c r="AL11" s="34"/>
       <c r="AM11" s="34"/>
       <c r="AN11" s="34"/>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>TEST AUTOMAZIONE PUNTI</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="24.0" customHeight="1">
       <c r="A12" s="35"/>
@@ -2009,9 +2013,7 @@
         <v>3</v>
       </c>
       <c r="W12" s="8"/>
-      <c r="X12" s="11"/>
       <c r="Y12" s="34"/>
-      <c r="Z12" s="34"/>
       <c r="AA12" s="34"/>
       <c r="AB12" s="34"/>
       <c r="AC12" s="34"/>
@@ -2026,6 +2028,14 @@
       <c r="AL12" s="34"/>
       <c r="AM12" s="34"/>
       <c r="AN12" s="34"/>
+      <c r="X12" s="1" t="inlineStr">
+        <is>
+          <t>Riga Poleman test</t>
+        </is>
+      </c>
+      <c r="Z12" s="1">
+        <v>3</v>
+      </c>
     </row>
     <row r="13" ht="24.0" customHeight="1">
       <c r="A13" s="47" t="s">
@@ -2052,29 +2062,32 @@
       </c>
       <c r="Q13" s="87" t="str">
         <f t="shared" ref="Q13:T13" si="2">Q7</f>
-        <v/>
+        <v>
+        </v>
       </c>
       <c r="R13" s="87" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>
+        </v>
       </c>
       <c r="S13" s="87" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>
+        </v>
       </c>
       <c r="T13" s="87" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>
+        </v>
       </c>
       <c r="U13" s="89"/>
       <c r="V13" s="88" t="str">
         <f>V7</f>
-        <v/>
+        <v>
+        </v>
       </c>
       <c r="W13" s="8"/>
-      <c r="X13" s="11"/>
       <c r="Y13" s="34"/>
-      <c r="Z13" s="34"/>
       <c r="AA13" s="34"/>
       <c r="AB13" s="34"/>
       <c r="AC13" s="34"/>
@@ -2089,6 +2102,16 @@
       <c r="AL13" s="34"/>
       <c r="AM13" s="34"/>
       <c r="AN13" s="34"/>
+      <c r="X13" s="1" t="inlineStr">
+        <is>
+          <t>Pole ufficiale</t>
+        </is>
+      </c>
+      <c r="Z13" s="1" t="inlineStr">
+        <is>
+          <t>Russell</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="24.0" customHeight="1">
       <c r="A14" s="49"/>
@@ -2136,9 +2159,7 @@
         <v>3</v>
       </c>
       <c r="W14" s="8"/>
-      <c r="X14" s="11"/>
       <c r="Y14" s="34"/>
-      <c r="Z14" s="34"/>
       <c r="AA14" s="34"/>
       <c r="AB14" s="34"/>
       <c r="AC14" s="34"/>
@@ -2153,6 +2174,16 @@
       <c r="AL14" s="34"/>
       <c r="AM14" s="34"/>
       <c r="AN14" s="34"/>
+      <c r="X14" s="1" t="inlineStr">
+        <is>
+          <t>1Â° ufficiale</t>
+        </is>
+      </c>
+      <c r="Z14" s="1" t="inlineStr">
+        <is>
+          <t>Russell</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="24.0" customHeight="1">
       <c r="A15" s="81" t="s">
@@ -2181,9 +2212,7 @@
       <c r="U15" s="11"/>
       <c r="V15" s="11"/>
       <c r="W15" s="8"/>
-      <c r="X15" s="11"/>
       <c r="Y15" s="34"/>
-      <c r="Z15" s="34"/>
       <c r="AA15" s="34"/>
       <c r="AB15" s="34"/>
       <c r="AC15" s="34"/>
@@ -2198,6 +2227,16 @@
       <c r="AL15" s="34"/>
       <c r="AM15" s="34"/>
       <c r="AN15" s="34"/>
+      <c r="X15" s="1" t="inlineStr">
+        <is>
+          <t>2Â° ufficiale</t>
+        </is>
+      </c>
+      <c r="Z15" s="1" t="inlineStr">
+        <is>
+          <t>Antonelli</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="24.0" customHeight="1">
       <c r="A16" s="35"/>
@@ -2224,9 +2263,7 @@
       <c r="U16" s="11"/>
       <c r="V16" s="11"/>
       <c r="W16" s="8"/>
-      <c r="X16" s="11"/>
       <c r="Y16" s="34"/>
-      <c r="Z16" s="34"/>
       <c r="AA16" s="34"/>
       <c r="AB16" s="34"/>
       <c r="AC16" s="34"/>
@@ -2241,6 +2278,16 @@
       <c r="AL16" s="34"/>
       <c r="AM16" s="34"/>
       <c r="AN16" s="34"/>
+      <c r="X16" s="1" t="inlineStr">
+        <is>
+          <t>3Â° ufficiale</t>
+        </is>
+      </c>
+      <c r="Z16" s="1" t="inlineStr">
+        <is>
+          <t>Leclerc</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="24.0" customHeight="1">
       <c r="A17" s="94" t="s">
@@ -2312,15 +2359,8 @@
       <c r="U18" s="11"/>
       <c r="V18" s="11"/>
       <c r="W18" s="8"/>
-      <c r="X18" s="11"/>
       <c r="Y18" s="34"/>
       <c r="Z18" s="34"/>
-      <c r="AA18" s="34"/>
-      <c r="AB18" s="34"/>
-      <c r="AC18" s="34"/>
-      <c r="AD18" s="34"/>
-      <c r="AE18" s="34"/>
-      <c r="AF18" s="34"/>
       <c r="AG18" s="34"/>
       <c r="AH18" s="34"/>
       <c r="AI18" s="34"/>
@@ -2329,6 +2369,41 @@
       <c r="AL18" s="34"/>
       <c r="AM18" s="34"/>
       <c r="AN18" s="34"/>
+      <c r="X18" s="2" t="inlineStr">
+        <is>
+          <t>Punteggio test</t>
+        </is>
+      </c>
+      <c r="AA18" s="1" t="inlineStr">
+        <is>
+          <t>Andrea</t>
+        </is>
+      </c>
+      <c r="AB18" s="1" t="inlineStr">
+        <is>
+          <t>Giovanni</t>
+        </is>
+      </c>
+      <c r="AC18" s="1" t="inlineStr">
+        <is>
+          <t>Luca</t>
+        </is>
+      </c>
+      <c r="AD18" s="1" t="inlineStr">
+        <is>
+          <t>Marco</t>
+        </is>
+      </c>
+      <c r="AE18" s="1" t="inlineStr">
+        <is>
+          <t>Michele</t>
+        </is>
+      </c>
+      <c r="AF18" s="1" t="inlineStr">
+        <is>
+          <t>Salvo</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="24.0" customHeight="1">
       <c r="A19" s="81" t="s">
@@ -2358,15 +2433,8 @@
       <c r="U19" s="11"/>
       <c r="V19" s="11"/>
       <c r="W19" s="8"/>
-      <c r="X19" s="11"/>
       <c r="Y19" s="34"/>
       <c r="Z19" s="34"/>
-      <c r="AA19" s="34"/>
-      <c r="AB19" s="34"/>
-      <c r="AC19" s="34"/>
-      <c r="AD19" s="34"/>
-      <c r="AE19" s="34"/>
-      <c r="AF19" s="34"/>
       <c r="AG19" s="34"/>
       <c r="AH19" s="34"/>
       <c r="AI19" s="34"/>
@@ -2375,6 +2443,35 @@
       <c r="AL19" s="34"/>
       <c r="AM19" s="34"/>
       <c r="AN19" s="34"/>
+      <c r="X19" s="1" t="inlineStr">
+        <is>
+          <t>Totale</t>
+        </is>
+      </c>
+      <c r="AA19" s="1">
+        <f>IF(INDEX($C:$H,$Z$12,COLUMN()-26)=$Z$13,2,0)+IF(INDEX($C:$H,$Z$12+1,COLUMN()-26)=$Z$14,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+1,COLUMN()-26))&gt;0,1,0))+IF(INDEX($C:$H,$Z$12+2,COLUMN()-26)=$Z$15,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+2,COLUMN()-26))&gt;0,1,0))+IF(INDEX($C:$H,$Z$12+3,COLUMN()-26)=$Z$16,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+3,COLUMN()-26))&gt;0,1,0))</f>
+        <v>6</v>
+      </c>
+      <c r="AB19" s="1">
+        <f>IF(INDEX($C:$H,$Z$12,COLUMN()-26)=$Z$13,2,0)+IF(INDEX($C:$H,$Z$12+1,COLUMN()-26)=$Z$14,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+1,COLUMN()-26))&gt;0,1,0))+IF(INDEX($C:$H,$Z$12+2,COLUMN()-26)=$Z$15,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+2,COLUMN()-26))&gt;0,1,0))+IF(INDEX($C:$H,$Z$12+3,COLUMN()-26)=$Z$16,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+3,COLUMN()-26))&gt;0,1,0))</f>
+        <v>4</v>
+      </c>
+      <c r="AC19" s="1">
+        <f>IF(INDEX($C:$H,$Z$12,COLUMN()-26)=$Z$13,2,0)+IF(INDEX($C:$H,$Z$12+1,COLUMN()-26)=$Z$14,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+1,COLUMN()-26))&gt;0,1,0))+IF(INDEX($C:$H,$Z$12+2,COLUMN()-26)=$Z$15,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+2,COLUMN()-26))&gt;0,1,0))+IF(INDEX($C:$H,$Z$12+3,COLUMN()-26)=$Z$16,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+3,COLUMN()-26))&gt;0,1,0))</f>
+        <v>6</v>
+      </c>
+      <c r="AD19" s="1">
+        <f>IF(INDEX($C:$H,$Z$12,COLUMN()-26)=$Z$13,2,0)+IF(INDEX($C:$H,$Z$12+1,COLUMN()-26)=$Z$14,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+1,COLUMN()-26))&gt;0,1,0))+IF(INDEX($C:$H,$Z$12+2,COLUMN()-26)=$Z$15,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+2,COLUMN()-26))&gt;0,1,0))+IF(INDEX($C:$H,$Z$12+3,COLUMN()-26)=$Z$16,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+3,COLUMN()-26))&gt;0,1,0))</f>
+        <v>6</v>
+      </c>
+      <c r="AE19" s="1">
+        <f>IF(INDEX($C:$H,$Z$12,COLUMN()-26)=$Z$13,2,0)+IF(INDEX($C:$H,$Z$12+1,COLUMN()-26)=$Z$14,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+1,COLUMN()-26))&gt;0,1,0))+IF(INDEX($C:$H,$Z$12+2,COLUMN()-26)=$Z$15,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+2,COLUMN()-26))&gt;0,1,0))+IF(INDEX($C:$H,$Z$12+3,COLUMN()-26)=$Z$16,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+3,COLUMN()-26))&gt;0,1,0))</f>
+        <v>2</v>
+      </c>
+      <c r="AF19" s="1">
+        <f>IF(INDEX($C:$H,$Z$12,COLUMN()-26)=$Z$13,2,0)+IF(INDEX($C:$H,$Z$12+1,COLUMN()-26)=$Z$14,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+1,COLUMN()-26))&gt;0,1,0))+IF(INDEX($C:$H,$Z$12+2,COLUMN()-26)=$Z$15,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+2,COLUMN()-26))&gt;0,1,0))+IF(INDEX($C:$H,$Z$12+3,COLUMN()-26)=$Z$16,3,IF(COUNTIF($Z$14:$Z$16,INDEX($C:$H,$Z$12+3,COLUMN()-26))&gt;0,1,0))</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="20" ht="24.0" customHeight="1">
       <c r="A20" s="35"/>
@@ -2402,9 +2499,7 @@
       <c r="U20" s="11"/>
       <c r="V20" s="11"/>
       <c r="W20" s="8"/>
-      <c r="X20" s="11"/>
       <c r="Y20" s="34"/>
-      <c r="Z20" s="34"/>
       <c r="AA20" s="34"/>
       <c r="AB20" s="34"/>
       <c r="AC20" s="34"/>
@@ -2419,6 +2514,16 @@
       <c r="AL20" s="34"/>
       <c r="AM20" s="34"/>
       <c r="AN20" s="34"/>
+      <c r="X20" s="1" t="inlineStr">
+        <is>
+          <t>Regola</t>
+        </is>
+      </c>
+      <c r="Z20" s="1" t="inlineStr">
+        <is>
+          <t>Pole=2, esatta=3, podio=1</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="24.0" customHeight="1">
       <c r="A21" s="94" t="s">

</xml_diff>